<commit_message>
Updated CAN_grids model - 2025-09-17 02:36
</commit_message>
<xml_diff>
--- a/VerveStacks_CAN_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_CAN_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CAN_grids\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8D65B563-282F-428A-B6B5-23FE133D61A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE8EC1EE-E12B-46D0-B3B4-091E19B98F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3675" yWindow="3675" windowWidth="21600" windowHeight="12683" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="368" yWindow="368" windowWidth="21599" windowHeight="12682" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AVA" sheetId="6" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated CAN_grids model - 2025-09-17 10:05
</commit_message>
<xml_diff>
--- a/VerveStacks_CAN_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_CAN_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CAN_grids\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE8EC1EE-E12B-46D0-B3B4-091E19B98F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8BE6A2AE-C376-498B-B16E-3D3A83C1BC01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="368" yWindow="368" windowWidth="21599" windowHeight="12682" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AVA" sheetId="6" r:id="rId1"/>

</xml_diff>